<commit_message>
Fix subcategory dropdown not showing on Windows Excel
Windows Excel enforces a 255-character limit on inline data validation
source strings. The fitting subcategory list (34 items) exceeded this
limit, causing the dropdown to silently fail on Windows while working
fine on Mac.

Fix: put subcategories on a hidden 'Lists' sheet inside the workbook
and reference it as a range (Lists!$A$1:$A$34) instead of an inline
comma-separated string. Range references have no character limit on
any platform.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Items-Fitting.xlsx
+++ b/public/Items-Fitting.xlsx
@@ -13,6 +13,7 @@
   </bookViews>
   <sheets>
     <sheet name="Fitting Items" sheetId="1" r:id="rId1"/>
+    <sheet name="Lists" sheetId="2" r:id="rId5" state="hidden"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -72,6 +73,102 @@
   </si>
   <si>
     <t xml:space="preserve">202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ball_with_nut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thali_base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">l_drop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stopper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_lock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hinges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">balustred_cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">baluster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">master_pillar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">starwindow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">butterfly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gamla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">baind</t>
+  </si>
+  <si>
+    <t xml:space="preserve">star_ring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bhala</t>
+  </si>
+  <si>
+    <t xml:space="preserve">braket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ground_braket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">om</t>
+  </si>
+  <si>
+    <t xml:space="preserve">swastik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shubh_labh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mel_femel_nut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gate_wheel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gate_opener</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kancha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">besh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pendi</t>
   </si>
 </sst>
 </file>
@@ -575,7 +672,7 @@
   </sheetData>
   <dataValidations>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="A2:A1000">
-      <formula1>"ball,ball_with_nut,base,thali_base,cap,bush,l_drop,stopper,d_lock,hinges,balustred_cap,baluster,master_pillar,starwindow,butterfly,gamla,step,baind,star_ring,ring,bhala,braket,ground_braket,om,swastik,shubh_labh,mel_femel_nut,flower,bail,gate_wheel,gate_opener,kancha,besh,pendi"</formula1>
+      <formula1>Lists!$A$1:$A$34</formula1>
       <formula2/>
     </dataValidation>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="B2:B1000">
@@ -589,4 +686,182 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add new fitting subcategories and type options
New subcategories: band, shubh, ganesh, lock_kunda
Also add kancha/besh/pendi to ItemForm (were missing from frontend only)

New type options in Excel dropdown: Half, Full, One Side, Two Side,
Half Plate, Full Plate, Dibbi, Non Dibbi, Two Pin, Three Pin
(in addition to existing Round/Square)

Subcategory-type mapping:
- band → Half / Full
- kancha → One Side / Two Side
- shubh / swastik / ganesh / om → Half Plate / Full Plate
- butterfly → Dibbi / Non Dibbi
- bush → Two Pin / Three Pin

Updated: models enum, ItemForm, inventory page filters,
Excel scripts, regenerated Items-Fitting.xlsx and Sales-Fitting.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Items-Fitting.xlsx
+++ b/public/Items-Fitting.xlsx
@@ -81,30 +81,60 @@
     <t xml:space="preserve">base</t>
   </si>
   <si>
+    <t xml:space="preserve">Half</t>
+  </si>
+  <si>
     <t xml:space="preserve">thali_base</t>
   </si>
   <si>
+    <t xml:space="preserve">Full</t>
+  </si>
+  <si>
     <t xml:space="preserve">cap</t>
   </si>
   <si>
+    <t xml:space="preserve">One Side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two Side</t>
+  </si>
+  <si>
     <t xml:space="preserve">l_drop</t>
   </si>
   <si>
+    <t xml:space="preserve">Half Plate</t>
+  </si>
+  <si>
     <t xml:space="preserve">stopper</t>
   </si>
   <si>
+    <t xml:space="preserve">Full Plate</t>
+  </si>
+  <si>
     <t xml:space="preserve">d_lock</t>
   </si>
   <si>
+    <t xml:space="preserve">Dibbi</t>
+  </si>
+  <si>
     <t xml:space="preserve">hinges</t>
   </si>
   <si>
+    <t xml:space="preserve">Non Dibbi</t>
+  </si>
+  <si>
     <t xml:space="preserve">balustred_cap</t>
   </si>
   <si>
+    <t xml:space="preserve">Two Pin</t>
+  </si>
+  <si>
     <t xml:space="preserve">baluster</t>
   </si>
   <si>
+    <t xml:space="preserve">Three Pin</t>
+  </si>
+  <si>
     <t xml:space="preserve">master_pillar</t>
   </si>
   <si>
@@ -147,6 +177,9 @@
     <t xml:space="preserve">shubh_labh</t>
   </si>
   <si>
+    <t xml:space="preserve">shubh</t>
+  </si>
+  <si>
     <t xml:space="preserve">mel_femel_nut</t>
   </si>
   <si>
@@ -169,6 +202,15 @@
   </si>
   <si>
     <t xml:space="preserve">pendi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ganesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lock_kunda</t>
   </si>
 </sst>
 </file>
@@ -672,11 +714,11 @@
   </sheetData>
   <dataValidations>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="A2:A1000">
-      <formula1>Lists!$A$1:$A$34</formula1>
+      <formula1>Lists!$A$1:$A$38</formula1>
       <formula2/>
     </dataValidation>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="B2:B1000">
-      <formula1>"Round,Square"</formula1>
+      <formula1>Lists!$B$1:$B$12</formula1>
       <formula2/>
     </dataValidation>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="D2:D1000">
@@ -696,170 +738,226 @@
       <c r="A1" t="s">
         <v>8</v>
       </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>12</v>
       </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new fitting subcategories, types, and re-add additional charges label
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Items-Fitting.xlsx
+++ b/public/Items-Fitting.xlsx
@@ -138,21 +138,39 @@
     <t xml:space="preserve">master_pillar</t>
   </si>
   <si>
+    <t xml:space="preserve">Ring</t>
+  </si>
+  <si>
     <t xml:space="preserve">starwindow</t>
   </si>
   <si>
+    <t xml:space="preserve">Varasi</t>
+  </si>
+  <si>
     <t xml:space="preserve">butterfly</t>
   </si>
   <si>
+    <t xml:space="preserve">Rassi</t>
+  </si>
+  <si>
     <t xml:space="preserve">gamla</t>
   </si>
   <si>
+    <t xml:space="preserve">Double Wall</t>
+  </si>
+  <si>
     <t xml:space="preserve">step</t>
   </si>
   <si>
+    <t xml:space="preserve">Matka</t>
+  </si>
+  <si>
     <t xml:space="preserve">baind</t>
   </si>
   <si>
+    <t xml:space="preserve">Rectangle</t>
+  </si>
+  <si>
     <t xml:space="preserve">star_ring</t>
   </si>
   <si>
@@ -211,6 +229,24 @@
   </si>
   <si>
     <t xml:space="preserve">lock_kunda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trishul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">umbrella_wall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kalash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">janzeer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jhula_set</t>
   </si>
 </sst>
 </file>
@@ -714,11 +750,11 @@
   </sheetData>
   <dataValidations>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="A2:A1000">
-      <formula1>Lists!$A$1:$A$38</formula1>
+      <formula1>Lists!$A$1:$A$44</formula1>
       <formula2/>
     </dataValidation>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="B2:B1000">
-      <formula1>Lists!$B$1:$B$12</formula1>
+      <formula1>Lists!$B$1:$B$18</formula1>
       <formula2/>
     </dataValidation>
     <dataValidation type="list" allowBlank="true" showInputMessage="undefined" prompt="undefined" promptTitle="undefined" showErrorMessage="undefined" error="undefined" errorTitle="undefined" operator="undefined" sqref="D2:D1000">
@@ -834,130 +870,178 @@
       <c r="A13" t="s">
         <v>36</v>
       </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>46</v>
+      </c>
+      <c r="B18" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>61</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>